<commit_message>
Rombak premium: 21 program, ikon SVG, pratinjau dashboard, 2 workbook baru
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ATKdQjtjDkbCW8CD6F26vC
</commit_message>
<xml_diff>
--- a/demo-excel/02-Aging-Piutang-Utang-demo.xlsx
+++ b/demo-excel/02-Aging-Piutang-Utang-demo.xlsx
@@ -352,7 +352,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Total Pelanggan per Kelompok Umur (Rp)</a:t>
+              <a:t>Total Pelanggan per Kelompok Umur (Rp juta)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -366,7 +366,13 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0EA5A4"/>
+            </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="0EA5A4"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -390,6 +396,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -401,8 +408,19 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="E3E8F1"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0,," sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -423,7 +441,7 @@
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="2880000"/>
+    <ext cx="5760000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>